<commit_message>
sync excel/2026/实时现货_用电侧小时电价.xlsx from private
</commit_message>
<xml_diff>
--- a/excel/2026/实时现货_用电侧小时电价.xlsx
+++ b/excel/2026/实时现货_用电侧小时电价.xlsx
@@ -1194,7 +1194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z289"/>
+  <dimension ref="A1:Z294"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:26">
@@ -24194,6 +24194,391 @@
         <v>83.36</v>
       </c>
     </row>
+    <row r="290" spans="1:26">
+      <c r="A290" s="2">
+        <v>46310</v>
+      </c>
+      <c r="C290">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="D290">
+        <v>0</v>
+      </c>
+      <c r="E290">
+        <v>-2.51</v>
+      </c>
+      <c r="F290">
+        <v>0</v>
+      </c>
+      <c r="G290">
+        <v>196.92</v>
+      </c>
+      <c r="H290">
+        <v>400.01</v>
+      </c>
+      <c r="I290">
+        <v>393.57</v>
+      </c>
+      <c r="J290">
+        <v>221.38</v>
+      </c>
+      <c r="K290">
+        <v>202.5</v>
+      </c>
+      <c r="L290">
+        <v>354.07</v>
+      </c>
+      <c r="M290">
+        <v>304.94</v>
+      </c>
+      <c r="N290">
+        <v>262.77</v>
+      </c>
+      <c r="O290">
+        <v>49.18</v>
+      </c>
+      <c r="P290">
+        <v>119.58</v>
+      </c>
+      <c r="Q290">
+        <v>364.14</v>
+      </c>
+      <c r="R290">
+        <v>486.36</v>
+      </c>
+      <c r="S290">
+        <v>522.96</v>
+      </c>
+      <c r="T290">
+        <v>506.15</v>
+      </c>
+      <c r="U290">
+        <v>496.22</v>
+      </c>
+      <c r="V290">
+        <v>506.58</v>
+      </c>
+      <c r="W290">
+        <v>503.35</v>
+      </c>
+      <c r="X290">
+        <v>491.2</v>
+      </c>
+      <c r="Y290">
+        <v>494.86</v>
+      </c>
+      <c r="Z290">
+        <v>497.25</v>
+      </c>
+    </row>
+    <row r="291" spans="1:26">
+      <c r="A291" s="2">
+        <v>46311</v>
+      </c>
+      <c r="C291">
+        <v>492.92</v>
+      </c>
+      <c r="D291">
+        <v>492.21</v>
+      </c>
+      <c r="E291">
+        <v>493.51</v>
+      </c>
+      <c r="F291">
+        <v>493.17</v>
+      </c>
+      <c r="G291">
+        <v>493.59</v>
+      </c>
+      <c r="H291">
+        <v>496.69</v>
+      </c>
+      <c r="I291">
+        <v>495.98</v>
+      </c>
+      <c r="J291">
+        <v>480.2</v>
+      </c>
+      <c r="K291">
+        <v>443.01</v>
+      </c>
+      <c r="L291">
+        <v>264.1</v>
+      </c>
+      <c r="M291">
+        <v>42.64</v>
+      </c>
+      <c r="N291">
+        <v>-19.95</v>
+      </c>
+      <c r="O291">
+        <v>-59.85</v>
+      </c>
+      <c r="P291">
+        <v>384.66</v>
+      </c>
+      <c r="Q291">
+        <v>417.09</v>
+      </c>
+      <c r="R291">
+        <v>465.66</v>
+      </c>
+      <c r="S291">
+        <v>482.22</v>
+      </c>
+      <c r="T291">
+        <v>475.73</v>
+      </c>
+      <c r="U291">
+        <v>467.75</v>
+      </c>
+      <c r="V291">
+        <v>472.16</v>
+      </c>
+      <c r="W291">
+        <v>471.88</v>
+      </c>
+      <c r="X291">
+        <v>474.9</v>
+      </c>
+      <c r="Y291">
+        <v>482.28</v>
+      </c>
+      <c r="Z291">
+        <v>463.19</v>
+      </c>
+    </row>
+    <row r="292" spans="1:26">
+      <c r="A292" s="2">
+        <v>46312</v>
+      </c>
+      <c r="C292">
+        <v>454.11</v>
+      </c>
+      <c r="D292">
+        <v>441.48</v>
+      </c>
+      <c r="E292">
+        <v>425.97</v>
+      </c>
+      <c r="F292">
+        <v>413.52</v>
+      </c>
+      <c r="G292">
+        <v>400.17</v>
+      </c>
+      <c r="H292">
+        <v>383.45</v>
+      </c>
+      <c r="I292">
+        <v>317.67</v>
+      </c>
+      <c r="J292">
+        <v>285.89</v>
+      </c>
+      <c r="K292">
+        <v>379</v>
+      </c>
+      <c r="L292">
+        <v>404.89</v>
+      </c>
+      <c r="M292">
+        <v>443.42</v>
+      </c>
+      <c r="N292">
+        <v>461.63</v>
+      </c>
+      <c r="O292">
+        <v>467.1</v>
+      </c>
+      <c r="P292">
+        <v>486.13</v>
+      </c>
+      <c r="Q292">
+        <v>483.13</v>
+      </c>
+      <c r="R292">
+        <v>458.39</v>
+      </c>
+      <c r="S292">
+        <v>421.31</v>
+      </c>
+      <c r="T292">
+        <v>445.37</v>
+      </c>
+      <c r="U292">
+        <v>418.49</v>
+      </c>
+      <c r="V292">
+        <v>431.86</v>
+      </c>
+      <c r="W292">
+        <v>440.06</v>
+      </c>
+      <c r="X292">
+        <v>419.25</v>
+      </c>
+      <c r="Y292">
+        <v>429.29</v>
+      </c>
+      <c r="Z292">
+        <v>405.1</v>
+      </c>
+    </row>
+    <row r="293" spans="1:26">
+      <c r="A293" s="2">
+        <v>46313</v>
+      </c>
+      <c r="C293">
+        <v>452.48</v>
+      </c>
+      <c r="D293">
+        <v>433.22</v>
+      </c>
+      <c r="E293">
+        <v>397.56</v>
+      </c>
+      <c r="F293">
+        <v>363.45</v>
+      </c>
+      <c r="G293">
+        <v>81.55</v>
+      </c>
+      <c r="H293">
+        <v>21.85</v>
+      </c>
+      <c r="I293">
+        <v>69.29000000000001</v>
+      </c>
+      <c r="J293">
+        <v>-21.43</v>
+      </c>
+      <c r="K293">
+        <v>-80</v>
+      </c>
+      <c r="L293">
+        <v>-80</v>
+      </c>
+      <c r="M293">
+        <v>-80</v>
+      </c>
+      <c r="N293">
+        <v>-80</v>
+      </c>
+      <c r="O293">
+        <v>-80</v>
+      </c>
+      <c r="P293">
+        <v>-80</v>
+      </c>
+      <c r="Q293">
+        <v>-80</v>
+      </c>
+      <c r="R293">
+        <v>85.70999999999999</v>
+      </c>
+      <c r="S293">
+        <v>547.13</v>
+      </c>
+      <c r="T293">
+        <v>516.11</v>
+      </c>
+      <c r="U293">
+        <v>496.21</v>
+      </c>
+      <c r="V293">
+        <v>504.74</v>
+      </c>
+      <c r="W293">
+        <v>507.84</v>
+      </c>
+      <c r="X293">
+        <v>509.13</v>
+      </c>
+      <c r="Y293">
+        <v>513.4299999999999</v>
+      </c>
+      <c r="Z293">
+        <v>501.33</v>
+      </c>
+    </row>
+    <row r="294" spans="1:26">
+      <c r="A294" s="2">
+        <v>46314</v>
+      </c>
+      <c r="C294">
+        <v>466.03</v>
+      </c>
+      <c r="D294">
+        <v>462.74</v>
+      </c>
+      <c r="E294">
+        <v>465.68</v>
+      </c>
+      <c r="F294">
+        <v>467.83</v>
+      </c>
+      <c r="G294">
+        <v>467.04</v>
+      </c>
+      <c r="H294">
+        <v>467.56</v>
+      </c>
+      <c r="I294">
+        <v>467.48</v>
+      </c>
+      <c r="J294">
+        <v>460.6</v>
+      </c>
+      <c r="K294">
+        <v>419.05</v>
+      </c>
+      <c r="L294">
+        <v>403.2</v>
+      </c>
+      <c r="M294">
+        <v>441.61</v>
+      </c>
+      <c r="N294">
+        <v>468.32</v>
+      </c>
+      <c r="O294">
+        <v>463.63</v>
+      </c>
+      <c r="P294">
+        <v>468.92</v>
+      </c>
+      <c r="Q294">
+        <v>466.21</v>
+      </c>
+      <c r="R294">
+        <v>459.67</v>
+      </c>
+      <c r="S294">
+        <v>455.94</v>
+      </c>
+      <c r="T294">
+        <v>463.68</v>
+      </c>
+      <c r="U294">
+        <v>460.74</v>
+      </c>
+      <c r="V294">
+        <v>454.92</v>
+      </c>
+      <c r="W294">
+        <v>452.51</v>
+      </c>
+      <c r="X294">
+        <v>447.06</v>
+      </c>
+      <c r="Y294">
+        <v>453.53</v>
+      </c>
+      <c r="Z294">
+        <v>447.38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>